<commit_message>
Close the defect cross-reference loop
DEMO-7 (duplicate DOM ids) and DEMO-8 (trailing newline in a product title)
were reachable from the Defects tab but not from any test case row, so a reader
scanning the case sheets would never see them. Both now cite their defect, and
every one of the 15 is reachable in both directions.

Found by an integrity check over the generated data: defect IDs cited vs
defined, case IDs referenced by defect rows, duplicate IDs, and automation
references pointing at files that exist.

Claude-Session: https://claude.ai/code/session_01Y328Wm7ZEccLPDEo6HwUpR
</commit_message>
<xml_diff>
--- a/docs/DemoBlaze-Test-Cases.xlsx
+++ b/docs/DemoBlaze-Test-Cases.xlsx
@@ -7231,7 +7231,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="48" customHeight="1">
+    <row r="50" ht="62" customHeight="1">
       <c r="A50" s="21" t="inlineStr">
         <is>
           <t>CRT-049</t>
@@ -7275,7 +7275,7 @@
       </c>
       <c r="I50" s="22" t="inlineStr">
         <is>
-          <t>Each filter returns a non-empty set and no product from another category leaks in</t>
+          <t>Each filter returns a non-empty set and no product from another category leaks in. Note the three category links share id='itemc' (DEMO-7), so they must be selected by role and text</t>
         </is>
       </c>
       <c r="J50" s="23" t="inlineStr">
@@ -7288,13 +7288,13 @@
           <t>tests/api/catalog.api.spec.ts › filters by category without leaking other categories</t>
         </is>
       </c>
-      <c r="L50" s="22" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="62" customHeight="1">
+      <c r="L50" s="31" t="inlineStr">
+        <is>
+          <t>DEMO-7</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="76" customHeight="1">
       <c r="A51" s="24" t="inlineStr">
         <is>
           <t>CRT-050</t>
@@ -7338,7 +7338,7 @@
       </c>
       <c r="I51" s="25" t="inlineStr">
         <is>
-          <t>/entries returns only the first 9 of 15 products. Any test or client that treats it as the whole catalogue will miss every monitor — documented in docs/api-contract.md</t>
+          <t>/entries returns only the first 9 of 15 products. Any test or client that treats it as the whole catalogue will miss every monitor — documented in docs/api-contract.md. One title also carries a trailing newline (DEMO-8), so title comparisons must be trimmed</t>
         </is>
       </c>
       <c r="J51" s="27" t="inlineStr">
@@ -7351,9 +7351,9 @@
           <t>tests/api/catalog.api.spec.ts › returns a non-empty product list</t>
         </is>
       </c>
-      <c r="L51" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="L51" s="31" t="inlineStr">
+        <is>
+          <t>DEMO-8</t>
         </is>
       </c>
     </row>

</xml_diff>